<commit_message>
Add approximate T-S density contour controls and release documentation
- Add approximate σ0 contour controls to T-S pages 03 and 34.
- Document limitations, TEOS-10 follow-up plan, and citation/license checklist.
- Publish the zero-row User Excel sample and remove obsolete temporary files.
- Keep internal development-only files excluded from public repositories.
</commit_message>
<xml_diff>
--- a/local_data/user_data.xlsx
+++ b/local_data/user_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/toyoho/Documents/study/704-Python/Webアプリ_main134_20230513/Streamlit_EnvGeo2/envgeo_seawater_v130/local_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39C21ADF-46A7-E14D-9BC9-7FDD0AE770D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B6303EB-BD83-E64B-BDA3-A946C90A1A89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5080" yWindow="2800" windowWidth="38400" windowHeight="21100" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="USER_DATA" sheetId="8" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">USER_DATA!$A$1:$X$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">USER_DATA!$A$1:$V$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Station</t>
     <phoneticPr fontId="3"/>
@@ -110,36 +110,6 @@
     <phoneticPr fontId="3"/>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="ＭＳ Ｐゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-      </rPr>
-      <t>石村メモ</t>
-    </r>
-    <rPh sb="0" eb="2">
-      <t>イシムラ</t>
-    </rPh>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="ＭＳ Ｐゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-      </rPr>
-      <t>石村ラベル</t>
-    </r>
-    <rPh sb="0" eb="2">
-      <t>イシムラ</t>
-    </rPh>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
     <t>Vertical</t>
     <phoneticPr fontId="3"/>
   </si>
@@ -166,7 +136,7 @@
     <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
     <numFmt numFmtId="179" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="18">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -257,12 +227,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="ＭＳ Ｐゴシック"/>
-      <family val="3"/>
-      <charset val="128"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="ＭＳ Ｐゴシック"/>
@@ -462,7 +426,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
       <alignment vertical="center"/>
@@ -475,11 +439,11 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -516,7 +480,7 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="11" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -528,9 +492,9 @@
     <xf numFmtId="178" fontId="11" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="137">
     <cellStyle name="Normal_TF5_Water Sampling Log" xfId="135" xr:uid="{A0FCD193-A019-D24C-AAB3-50CA4A140839}"/>
@@ -1123,16 +1087,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>20818</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>72869</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>791146</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>10409</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>919785</xdr:colOff>
+      <xdr:colOff>721998</xdr:colOff>
       <xdr:row>32</xdr:row>
-      <xdr:rowOff>10409</xdr:rowOff>
+      <xdr:rowOff>124917</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1155,7 +1119,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="988933" y="4674017"/>
+          <a:off x="791146" y="4798934"/>
           <a:ext cx="17117491" cy="999344"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1503,7 +1467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02E8E13E-78E2-6248-8EFC-B9675F6691E1}">
-  <dimension ref="A1:X43"/>
+  <dimension ref="A1:V43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="12.6640625" style="1" bestFit="1" customWidth="1"/>
@@ -1527,14 +1491,12 @@
     <col min="20" max="20" width="10.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="18.33203125" style="1" customWidth="1"/>
     <col min="22" max="22" width="60.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="35.33203125" style="4" customWidth="1"/>
-    <col min="24" max="24" width="24.33203125" style="4" customWidth="1"/>
-    <col min="25" max="25" width="12.83203125" style="4"/>
-    <col min="26" max="26" width="13" style="4" customWidth="1"/>
-    <col min="27" max="16384" width="12.83203125" style="4"/>
+    <col min="23" max="23" width="12.83203125" style="4"/>
+    <col min="24" max="24" width="13" style="4" customWidth="1"/>
+    <col min="25" max="16384" width="12.83203125" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="1" customFormat="1">
+    <row r="1" spans="1:22" s="1" customFormat="1">
       <c r="A1" s="11" t="s">
         <v>9</v>
       </c>
@@ -1569,7 +1531,7 @@
         <v>5</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>16</v>
@@ -1587,28 +1549,22 @@
         <v>2</v>
       </c>
       <c r="R1" s="11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="S1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="U1" s="9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="V1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="W1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:24" s="10" customFormat="1" ht="15">
+    </row>
+    <row r="2" spans="1:22" s="10" customFormat="1" ht="15">
       <c r="A2" s="16"/>
       <c r="B2" s="16"/>
       <c r="C2" s="16"/>
@@ -1632,7 +1588,7 @@
       <c r="U2" s="16"/>
       <c r="V2" s="16"/>
     </row>
-    <row r="3" spans="1:24" s="10" customFormat="1">
+    <row r="3" spans="1:22" s="10" customFormat="1">
       <c r="A3" s="16"/>
       <c r="B3" s="16"/>
       <c r="C3" s="16"/>
@@ -1656,7 +1612,7 @@
       <c r="U3" s="16"/>
       <c r="V3" s="16"/>
     </row>
-    <row r="4" spans="1:24" s="10" customFormat="1">
+    <row r="4" spans="1:22" s="10" customFormat="1">
       <c r="A4" s="16"/>
       <c r="B4" s="16"/>
       <c r="C4" s="16"/>
@@ -1680,7 +1636,7 @@
       <c r="U4" s="16"/>
       <c r="V4" s="16"/>
     </row>
-    <row r="5" spans="1:24" s="10" customFormat="1">
+    <row r="5" spans="1:22" s="10" customFormat="1">
       <c r="A5" s="16"/>
       <c r="B5" s="16"/>
       <c r="C5" s="16"/>
@@ -1704,7 +1660,7 @@
       <c r="U5" s="16"/>
       <c r="V5" s="16"/>
     </row>
-    <row r="6" spans="1:24" s="10" customFormat="1">
+    <row r="6" spans="1:22" s="10" customFormat="1">
       <c r="A6" s="16"/>
       <c r="B6" s="16"/>
       <c r="C6" s="16"/>
@@ -1728,7 +1684,7 @@
       <c r="U6" s="16"/>
       <c r="V6" s="16"/>
     </row>
-    <row r="7" spans="1:24">
+    <row r="7" spans="1:22">
       <c r="A7" s="16"/>
       <c r="B7" s="16"/>
       <c r="C7" s="16"/>
@@ -1752,7 +1708,7 @@
       <c r="U7" s="16"/>
       <c r="V7" s="16"/>
     </row>
-    <row r="8" spans="1:24">
+    <row r="8" spans="1:22">
       <c r="A8" s="16"/>
       <c r="B8" s="16"/>
       <c r="C8" s="16"/>
@@ -1776,7 +1732,7 @@
       <c r="U8" s="16"/>
       <c r="V8" s="16"/>
     </row>
-    <row r="9" spans="1:24">
+    <row r="9" spans="1:22">
       <c r="A9" s="16"/>
       <c r="B9" s="16"/>
       <c r="C9" s="16"/>
@@ -1800,7 +1756,7 @@
       <c r="U9" s="16"/>
       <c r="V9" s="16"/>
     </row>
-    <row r="10" spans="1:24">
+    <row r="10" spans="1:22">
       <c r="A10" s="16"/>
       <c r="B10" s="16"/>
       <c r="C10" s="16"/>
@@ -1824,7 +1780,7 @@
       <c r="U10" s="16"/>
       <c r="V10" s="16"/>
     </row>
-    <row r="11" spans="1:24">
+    <row r="11" spans="1:22">
       <c r="A11" s="16"/>
       <c r="B11" s="16"/>
       <c r="C11" s="16"/>
@@ -1848,7 +1804,7 @@
       <c r="U11" s="16"/>
       <c r="V11" s="16"/>
     </row>
-    <row r="12" spans="1:24">
+    <row r="12" spans="1:22">
       <c r="A12" s="16"/>
       <c r="B12" s="16"/>
       <c r="C12" s="16"/>
@@ -1872,7 +1828,7 @@
       <c r="U12" s="16"/>
       <c r="V12" s="16"/>
     </row>
-    <row r="13" spans="1:24">
+    <row r="13" spans="1:22">
       <c r="A13" s="16"/>
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
@@ -1896,7 +1852,7 @@
       <c r="U13" s="16"/>
       <c r="V13" s="16"/>
     </row>
-    <row r="14" spans="1:24">
+    <row r="14" spans="1:22">
       <c r="A14" s="16"/>
       <c r="B14" s="16"/>
       <c r="C14" s="16"/>
@@ -1920,7 +1876,7 @@
       <c r="U14" s="16"/>
       <c r="V14" s="16"/>
     </row>
-    <row r="15" spans="1:24">
+    <row r="15" spans="1:22">
       <c r="A15" s="16"/>
       <c r="B15" s="16"/>
       <c r="C15" s="16"/>
@@ -1944,7 +1900,7 @@
       <c r="U15" s="16"/>
       <c r="V15" s="16"/>
     </row>
-    <row r="16" spans="1:24">
+    <row r="16" spans="1:22">
       <c r="A16" s="16"/>
       <c r="B16" s="16"/>
       <c r="C16" s="16"/>
@@ -2617,7 +2573,7 @@
       <c r="V43" s="16"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X1" xr:uid="{0253FD36-6E03-42A4-9659-F22DA23DE40C}"/>
+  <autoFilter ref="A1:V1" xr:uid="{0253FD36-6E03-42A4-9659-F22DA23DE40C}"/>
   <phoneticPr fontId="3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292" r:id="rId1"/>

</xml_diff>